<commit_message>
Retrait de « sans carte bancaire » : kits, textes, calendrier, couverture, voix coupées et 9 vidéos refaites
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XRiR3Ga39EKt9eeNc8DXDQ
</commit_message>
<xml_diff>
--- a/LIMO-video/calendrier/CALENDRIER-PUBLICATION-LIMO.xlsx
+++ b/LIMO-video/calendrier/CALENDRIER-PUBLICATION-LIMO.xlsx
@@ -642,7 +642,7 @@
 2️⃣ Tes relances sont dans ta tête
 3️⃣ Tes soirées partent dans l'administratif
 Laquelle te parle le plus ? Dis-le en commentaire 👇
-👉 Essai gratuit 14 jours, sans carte bancaire : lien en bio.</t>
+👉 Essai gratuit 14 jours : lien en bio.</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -700,7 +700,7 @@
 Ton collègue, lui, regarde un film 🍿
 Son secret : Limo prépare sa semaine (relances, rendez-vous, dossiers).
 Identifie le collègue qui bosse encore le dimanche 😅
-👉 Essai gratuit 14 jours, sans carte bancaire : lien en bio.</t>
+👉 Essai gratuit 14 jours : lien en bio.</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -756,7 +756,7 @@
         <is>
           <t>Pendant que tu hésites, ton concurrent rappelle tes vendeurs. 📞
 Le mandat ne se gagne pas pendant l'estimation : il se gagne au suivi.
-👉 Essai gratuit 14 jours, sans carte bancaire : lien en bio.</t>
+👉 Essai gratuit 14 jours : lien en bio.</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -814,7 +814,7 @@
 1 h d'administratif par jour = plus de 200 h par an.
 200 h, c'est des dizaines de rendez-vous vendeurs que tu ne fais pas.
 Limo s'occupe des relances, comptes rendus, annonces et suivi des dossiers.
-Dès 49 €/mois. 👉 Essai gratuit 14 jours, sans carte bancaire : lien en bio.</t>
+Dès 49 €/mois. 👉 Essai gratuit 14 jours : lien en bio.</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -870,7 +870,7 @@
         <is>
           <t>Salut conseiller immo 👋 C'est moi, le robot de Limo.
 Mon job : te soulager de tout ce qui n'est pas de la vente. Relances, fiches, annonces, dossiers… je m'en occupe.
-👉 Essai gratuit 14 jours, sans carte bancaire : lien en bio.</t>
+👉 Essai gratuit 14 jours : lien en bio.</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -926,7 +926,7 @@
         <is>
           <t>Tu vends des biens d'exception. Ton suivi doit l'être aussi ✨
 Estimation, annonce soignée, relances au bon moment : Limo, le bras droit du conseiller immo.
-👉 Essai gratuit 14 jours, sans carte bancaire : lien en bio.</t>
+👉 Essai gratuit 14 jours : lien en bio.</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -1024,7 +1024,7 @@
           <t>Conseiller immo, regarde ça 👀
 Tu demandes « rappelle-moi le bien de M. et Mme T. »… et tout ressort : documents, propriétaires, estimation, diagnostics.
 Pendant ce temps, Limo relance tes acquéreurs et ton diagnostiqueur.
-👉 Essai gratuit 14 jours, sans carte bancaire : lien en bio.</t>
+👉 Essai gratuit 14 jours : lien en bio.</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
@@ -1082,7 +1082,7 @@
 Quelques jours plus tard, un autre panneau était sur la maison. 💔
 Le mandat ne se perd pas pendant l'estimation. Il se perd après.
 Même les meilleurs conseillers oublient parfois. Limo, jamais.
-👉 Essai gratuit 14 jours, sans carte bancaire : lien en bio.</t>
+👉 Essai gratuit 14 jours : lien en bio.</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
@@ -1138,7 +1138,7 @@
         <is>
           <t>Combien de mandats as-tu perdus cette année… juste par manque de suivi ? 🤔
 Limo relance tes vendeurs au bon moment et garde tous tes dossiers à jour.
-👉 Essai gratuit 14 jours, sans carte bancaire : lien en bio.</t>
+👉 Essai gratuit 14 jours : lien en bio.</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
@@ -1195,7 +1195,7 @@
           <t>POV : ton collègue a l'air moins débordé que toi… et rentre plus tôt 😅
 Son secret ? Limo, le bras droit du conseiller immo.
 Tag le collègue qui a besoin de voir ça 👇
-👉 Essai gratuit 14 jours, sans carte bancaire : lien en bio.</t>
+👉 Essai gratuit 14 jours : lien en bio.</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
@@ -1251,7 +1251,7 @@
         <is>
           <t>3 h du matin. Tu te réveilles en sursaut : « J'ai rappelé Mme Martin ?! » 😱
 Avec Limo, tu dors tranquille : les relances sont suivies pour toi.
-👉 Essai gratuit 14 jours, sans carte bancaire : lien en bio.</t>
+👉 Essai gratuit 14 jours : lien en bio.</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
@@ -1307,7 +1307,7 @@
         <is>
           <t>Un chalet, une vue, un acquéreur qui attend la bonne annonce 🏔️
 Avec Limo, l'annonce est rédigée en 2 minutes et tes acquéreurs compatibles sont relancés.
-👉 Essai gratuit 14 jours, sans carte bancaire : lien en bio.</t>
+👉 Essai gratuit 14 jours : lien en bio.</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
@@ -1404,7 +1404,7 @@
         <is>
           <t>8 h : priorités prêtes. 10 h : compte rendu dicté, fiche créée. 14 h : annonce rédigée. 18 h : diagnostiqueur relancé, notaire servi.
 Et toi ? Tu as passé ta journée avec tes clients 🏡
-👉 Essai gratuit 14 jours, sans carte bancaire : lien en bio.</t>
+👉 Essai gratuit 14 jours : lien en bio.</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1461,7 +1461,7 @@
           <t>Tout ce que Limo fait pour toi, en une vidéo 🧰
 Relances, estimations, annonces, dossiers, avis, suivi acquéreurs… le bras droit du conseiller immo.
 Lequel tu utiliserais en premier ?
-👉 Essai gratuit 14 jours, sans carte bancaire : lien en bio.</t>
+👉 Essai gratuit 14 jours : lien en bio.</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1517,7 +1517,7 @@
         <is>
           <t>Les red flags d'une journée de conseiller immo 🚩
 Tu en coches combien ? Dis-le en commentaire 👇
-👉 Essai gratuit 14 jours, sans carte bancaire : lien en bio.</t>
+👉 Essai gratuit 14 jours : lien en bio.</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -1573,7 +1573,7 @@
         <is>
           <t>Ton CRM est plein… mais il dort 😴
 Limo te dit qui relancer, quand, et prépare le message pour toi.
-👉 Essai gratuit 14 jours, sans carte bancaire : lien en bio.</t>
+👉 Essai gratuit 14 jours : lien en bio.</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1629,7 +1629,7 @@
         <is>
           <t>Vrai ou faux ? Le robot de Limo répond à tes idées reçues 🤖
 Ta réponse en commentaire 👇
-👉 Essai gratuit 14 jours, sans carte bancaire : lien en bio.</t>
+👉 Essai gratuit 14 jours : lien en bio.</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
@@ -1686,7 +1686,7 @@
           <t>Le jour de la signature, on oublie tout le reste 🤝
 Les appels du soir, les relances, les compromis, les diagnostics…
 Ton métier, c'est ça. Limo s'occupe du reste, du mandat à la signature.
-👉 Essai gratuit 14 jours, sans carte bancaire : lien en bio.</t>
+👉 Essai gratuit 14 jours : lien en bio.</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
@@ -1783,7 +1783,7 @@
         <is>
           <t>Conseiller immo, surchargé ? 😮‍💨
 Limo est fait pour ça.
-👉 Essai gratuit 14 jours, sans carte bancaire : lien en bio.</t>
+👉 Essai gratuit 14 jours : lien en bio.</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr">
@@ -1839,7 +1839,7 @@
         <is>
           <t>Tes avis Google, ta meilleure vitrine ⭐
 Limo t'aide à demander l'avis au bon moment et à y répondre.
-👉 Essai gratuit 14 jours, sans carte bancaire : lien en bio.</t>
+👉 Essai gratuit 14 jours : lien en bio.</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
@@ -1894,7 +1894,7 @@
       <c r="G28" s="7" t="inlineStr">
         <is>
           <t>10 secondes pour comprendre Limo ⏱️
-👉 Essai gratuit 14 jours, sans carte bancaire : lien en bio.</t>
+👉 Essai gratuit 14 jours : lien en bio.</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr">
@@ -1950,7 +1950,7 @@
         <is>
           <t>Toi, tu décroches un mandat depuis ta voiture.
 Pendant ce temps, Limo envoie l'estimation à la vendeuse 📲
-👉 Essai gratuit 14 jours, sans carte bancaire : lien en bio.</t>
+👉 Essai gratuit 14 jours : lien en bio.</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
@@ -2005,7 +2005,7 @@
       <c r="G30" s="7" t="inlineStr">
         <is>
           <t>Le robot de Limo réagit à ta journée de conseiller 😂
-👉 Essai gratuit 14 jours, sans carte bancaire : lien en bio.</t>
+👉 Essai gratuit 14 jours : lien en bio.</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr">
@@ -2062,7 +2062,7 @@
           <t>Ton métier, c'est le terrain, l'humain, la signature.
 Le reste ? Limo s'en occupe.
 Limo, le bras droit du conseiller immo.
-👉 Essai gratuit 14 jours, sans carte bancaire : lien en bio.</t>
+👉 Essai gratuit 14 jours : lien en bio.</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">

</xml_diff>